<commit_message>
amend/correct results of previous release
</commit_message>
<xml_diff>
--- a/Documentation/VectoResults_3.2.0.925.xlsx
+++ b/Documentation/VectoResults_3.2.0.925.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="192">
   <si>
     <t># VECTO 3.2.0.925 - 13.07.2017 14:11</t>
   </si>
@@ -594,13 +594,19 @@
   </si>
   <si>
     <t>Undefined</t>
+  </si>
+  <si>
+    <t>3-0</t>
+  </si>
+  <si>
+    <t># VECTO 3.2.0.925 - 31.07.2017 08:50</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -608,8 +614,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -634,6 +647,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -647,7 +666,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -656,6 +675,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="16" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -936,17 +958,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:DX31"/>
+  <dimension ref="A1:DX73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
     <col min="5" max="9" width="0" hidden="1" customWidth="1"/>
     <col min="68" max="68" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="17.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="18" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="72" max="72" width="18" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:126" x14ac:dyDescent="0.25">
@@ -9897,7 +9920,3492 @@
         <v>9.5490999999999993</v>
       </c>
     </row>
+    <row r="35" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>191</v>
+      </c>
+      <c r="BQ35"/>
+    </row>
+    <row r="36" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3</v>
+      </c>
+      <c r="D36" t="s">
+        <v>4</v>
+      </c>
+      <c r="E36" t="s">
+        <v>5</v>
+      </c>
+      <c r="F36" t="s">
+        <v>6</v>
+      </c>
+      <c r="G36" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" t="s">
+        <v>8</v>
+      </c>
+      <c r="I36" t="s">
+        <v>9</v>
+      </c>
+      <c r="J36" t="s">
+        <v>10</v>
+      </c>
+      <c r="K36" t="s">
+        <v>11</v>
+      </c>
+      <c r="L36" t="s">
+        <v>12</v>
+      </c>
+      <c r="M36" t="s">
+        <v>13</v>
+      </c>
+      <c r="N36" t="s">
+        <v>14</v>
+      </c>
+      <c r="O36" t="s">
+        <v>15</v>
+      </c>
+      <c r="P36" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>17</v>
+      </c>
+      <c r="R36" t="s">
+        <v>18</v>
+      </c>
+      <c r="S36" t="s">
+        <v>19</v>
+      </c>
+      <c r="T36" t="s">
+        <v>20</v>
+      </c>
+      <c r="U36" t="s">
+        <v>21</v>
+      </c>
+      <c r="V36" t="s">
+        <v>22</v>
+      </c>
+      <c r="W36" t="s">
+        <v>23</v>
+      </c>
+      <c r="X36" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z36" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD36" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE36" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF36" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG36" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH36" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI36" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ36" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK36" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL36" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM36" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN36" t="s">
+        <v>40</v>
+      </c>
+      <c r="AO36" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP36" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ36" t="s">
+        <v>43</v>
+      </c>
+      <c r="AR36" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS36" t="s">
+        <v>45</v>
+      </c>
+      <c r="AT36" t="s">
+        <v>46</v>
+      </c>
+      <c r="AU36" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV36" t="s">
+        <v>48</v>
+      </c>
+      <c r="AW36" t="s">
+        <v>49</v>
+      </c>
+      <c r="AX36" t="s">
+        <v>50</v>
+      </c>
+      <c r="AY36" t="s">
+        <v>51</v>
+      </c>
+      <c r="AZ36" t="s">
+        <v>52</v>
+      </c>
+      <c r="BA36" t="s">
+        <v>53</v>
+      </c>
+      <c r="BB36" t="s">
+        <v>154</v>
+      </c>
+      <c r="BC36" t="s">
+        <v>155</v>
+      </c>
+      <c r="BD36" t="s">
+        <v>54</v>
+      </c>
+      <c r="BE36" t="s">
+        <v>55</v>
+      </c>
+      <c r="BF36" t="s">
+        <v>56</v>
+      </c>
+      <c r="BG36" t="s">
+        <v>57</v>
+      </c>
+      <c r="BH36" t="s">
+        <v>58</v>
+      </c>
+      <c r="BI36" t="s">
+        <v>59</v>
+      </c>
+      <c r="BJ36" t="s">
+        <v>60</v>
+      </c>
+      <c r="BK36" t="s">
+        <v>61</v>
+      </c>
+      <c r="BL36" t="s">
+        <v>62</v>
+      </c>
+      <c r="BM36" t="s">
+        <v>63</v>
+      </c>
+      <c r="BN36" t="s">
+        <v>64</v>
+      </c>
+      <c r="BO36" t="s">
+        <v>65</v>
+      </c>
+      <c r="BP36" t="s">
+        <v>66</v>
+      </c>
+      <c r="BQ36" t="s">
+        <v>67</v>
+      </c>
+      <c r="BR36" t="s">
+        <v>68</v>
+      </c>
+      <c r="BS36" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT36" t="s">
+        <v>70</v>
+      </c>
+      <c r="BU36" t="s">
+        <v>71</v>
+      </c>
+      <c r="BV36" t="s">
+        <v>72</v>
+      </c>
+      <c r="BW36" t="s">
+        <v>73</v>
+      </c>
+      <c r="BX36" t="s">
+        <v>74</v>
+      </c>
+      <c r="BY36" t="s">
+        <v>75</v>
+      </c>
+      <c r="BZ36" t="s">
+        <v>76</v>
+      </c>
+      <c r="CA36" t="s">
+        <v>77</v>
+      </c>
+      <c r="CB36" t="s">
+        <v>78</v>
+      </c>
+      <c r="CC36" t="s">
+        <v>79</v>
+      </c>
+      <c r="CD36" t="s">
+        <v>156</v>
+      </c>
+      <c r="CE36" t="s">
+        <v>157</v>
+      </c>
+      <c r="CF36" t="s">
+        <v>158</v>
+      </c>
+      <c r="CG36" t="s">
+        <v>159</v>
+      </c>
+      <c r="CH36" t="s">
+        <v>84</v>
+      </c>
+      <c r="CI36" t="s">
+        <v>85</v>
+      </c>
+      <c r="CJ36" t="s">
+        <v>86</v>
+      </c>
+      <c r="CK36" t="s">
+        <v>87</v>
+      </c>
+      <c r="CL36" t="s">
+        <v>88</v>
+      </c>
+      <c r="CM36" t="s">
+        <v>89</v>
+      </c>
+      <c r="CN36" t="s">
+        <v>90</v>
+      </c>
+      <c r="CO36" t="s">
+        <v>91</v>
+      </c>
+      <c r="CP36" t="s">
+        <v>92</v>
+      </c>
+      <c r="CQ36" t="s">
+        <v>93</v>
+      </c>
+      <c r="CR36" t="s">
+        <v>94</v>
+      </c>
+      <c r="CS36" t="s">
+        <v>95</v>
+      </c>
+      <c r="CT36" t="s">
+        <v>96</v>
+      </c>
+      <c r="CU36" t="s">
+        <v>97</v>
+      </c>
+      <c r="CV36" t="s">
+        <v>98</v>
+      </c>
+      <c r="CW36" t="s">
+        <v>99</v>
+      </c>
+      <c r="CX36" t="s">
+        <v>100</v>
+      </c>
+      <c r="CY36" t="s">
+        <v>101</v>
+      </c>
+      <c r="CZ36" t="s">
+        <v>102</v>
+      </c>
+      <c r="DA36" t="s">
+        <v>103</v>
+      </c>
+      <c r="DB36" t="s">
+        <v>104</v>
+      </c>
+      <c r="DC36" t="s">
+        <v>105</v>
+      </c>
+      <c r="DD36" t="s">
+        <v>106</v>
+      </c>
+      <c r="DE36" t="s">
+        <v>107</v>
+      </c>
+      <c r="DF36" t="s">
+        <v>108</v>
+      </c>
+      <c r="DG36" t="s">
+        <v>109</v>
+      </c>
+      <c r="DH36" t="s">
+        <v>110</v>
+      </c>
+      <c r="DI36" t="s">
+        <v>111</v>
+      </c>
+      <c r="DJ36" t="s">
+        <v>112</v>
+      </c>
+      <c r="DK36" t="s">
+        <v>113</v>
+      </c>
+      <c r="DL36" t="s">
+        <v>114</v>
+      </c>
+      <c r="DM36" t="s">
+        <v>115</v>
+      </c>
+      <c r="DN36" t="s">
+        <v>116</v>
+      </c>
+      <c r="DO36" t="s">
+        <v>117</v>
+      </c>
+      <c r="DP36" t="s">
+        <v>118</v>
+      </c>
+      <c r="DQ36" t="s">
+        <v>119</v>
+      </c>
+      <c r="DR36" t="s">
+        <v>120</v>
+      </c>
+      <c r="DS36" t="s">
+        <v>121</v>
+      </c>
+      <c r="DT36" t="s">
+        <v>122</v>
+      </c>
+      <c r="DU36" t="s">
+        <v>123</v>
+      </c>
+      <c r="DV36" t="s">
+        <v>124</v>
+      </c>
+      <c r="DW36" t="s">
+        <v>125</v>
+      </c>
+      <c r="DX36" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" t="s">
+        <v>175</v>
+      </c>
+      <c r="C37" t="s">
+        <v>144</v>
+      </c>
+      <c r="D37" t="s">
+        <v>130</v>
+      </c>
+      <c r="E37" t="s">
+        <v>131</v>
+      </c>
+      <c r="G37" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>4670</v>
+      </c>
+      <c r="J37">
+        <v>3020</v>
+      </c>
+      <c r="K37">
+        <v>9590</v>
+      </c>
+      <c r="L37" t="s">
+        <v>131</v>
+      </c>
+      <c r="M37" t="s">
+        <v>163</v>
+      </c>
+      <c r="N37" t="s">
+        <v>133</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
+        <v>600</v>
+      </c>
+      <c r="Q37">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>6871</v>
+      </c>
+      <c r="S37">
+        <v>1</v>
+      </c>
+      <c r="T37">
+        <v>1</v>
+      </c>
+      <c r="U37">
+        <v>1</v>
+      </c>
+      <c r="V37">
+        <v>0</v>
+      </c>
+      <c r="W37">
+        <v>1</v>
+      </c>
+      <c r="X37">
+        <v>1</v>
+      </c>
+      <c r="Z37">
+        <v>4.83</v>
+      </c>
+      <c r="AA37">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AB37">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AC37">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD37">
+        <v>1</v>
+      </c>
+      <c r="AE37">
+        <v>1</v>
+      </c>
+      <c r="AF37">
+        <v>0</v>
+      </c>
+      <c r="AG37" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH37" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI37" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ37">
+        <v>1.35</v>
+      </c>
+      <c r="AK37">
+        <v>0.73</v>
+      </c>
+      <c r="AN37" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO37" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP37" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ37" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR37" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS37" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT37" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU37" t="s">
+        <v>176</v>
+      </c>
+      <c r="AV37">
+        <v>5.8</v>
+      </c>
+      <c r="BE37">
+        <v>3199.6950999999999</v>
+      </c>
+      <c r="BF37">
+        <v>27.815999999999999</v>
+      </c>
+      <c r="BG37">
+        <v>31.295999999999999</v>
+      </c>
+      <c r="BH37">
+        <v>-1.5800000000000002E-2</v>
+      </c>
+      <c r="BI37">
+        <v>5666.1364000000003</v>
+      </c>
+      <c r="BJ37">
+        <v>181.05</v>
+      </c>
+      <c r="BK37">
+        <v>5666.1364000000003</v>
+      </c>
+      <c r="BL37">
+        <v>181.05</v>
+      </c>
+      <c r="BM37">
+        <v>5666.1364000000003</v>
+      </c>
+      <c r="BN37">
+        <v>181.05</v>
+      </c>
+      <c r="BO37">
+        <v>5666.1364000000003</v>
+      </c>
+      <c r="BP37">
+        <v>181.05</v>
+      </c>
+      <c r="BQ37">
+        <v>5666.1364000000003</v>
+      </c>
+      <c r="BR37">
+        <v>181.05</v>
+      </c>
+      <c r="BS37" s="2">
+        <v>21.656700000000001</v>
+      </c>
+      <c r="BT37">
+        <v>7.1711</v>
+      </c>
+      <c r="BV37">
+        <v>566.68640000000005</v>
+      </c>
+      <c r="BW37">
+        <v>187.64449999999999</v>
+      </c>
+      <c r="BY37">
+        <v>21.1586</v>
+      </c>
+      <c r="BZ37">
+        <v>26.1282</v>
+      </c>
+      <c r="CA37">
+        <v>23.222899999999999</v>
+      </c>
+      <c r="CB37">
+        <v>1.1702999999999999</v>
+      </c>
+      <c r="CC37">
+        <v>0</v>
+      </c>
+      <c r="CD37">
+        <v>0</v>
+      </c>
+      <c r="CE37">
+        <v>3.1463999999999999</v>
+      </c>
+      <c r="CI37">
+        <v>3.1463999999999999</v>
+      </c>
+      <c r="CJ37">
+        <v>0</v>
+      </c>
+      <c r="CK37">
+        <v>0.47039999999999998</v>
+      </c>
+      <c r="CL37">
+        <v>0.1477</v>
+      </c>
+      <c r="CM37">
+        <v>0.55620000000000003</v>
+      </c>
+      <c r="CN37">
+        <v>0</v>
+      </c>
+      <c r="CO37">
+        <v>0</v>
+      </c>
+      <c r="CP37">
+        <v>0.42159999999999997</v>
+      </c>
+      <c r="CQ37">
+        <v>6.7967000000000004</v>
+      </c>
+      <c r="CR37">
+        <v>0</v>
+      </c>
+      <c r="CS37">
+        <v>5.3536000000000001</v>
+      </c>
+      <c r="CT37">
+        <v>5.3079000000000001</v>
+      </c>
+      <c r="CU37">
+        <v>-1E-4</v>
+      </c>
+      <c r="CV37">
+        <v>0</v>
+      </c>
+      <c r="CW37">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="CX37">
+        <v>-0.82699999999999996</v>
+      </c>
+      <c r="CY37">
+        <v>15.994999999999999</v>
+      </c>
+      <c r="CZ37">
+        <v>12.920500000000001</v>
+      </c>
+      <c r="DA37">
+        <v>51.113799999999998</v>
+      </c>
+      <c r="DB37">
+        <v>85</v>
+      </c>
+      <c r="DC37">
+        <v>1</v>
+      </c>
+      <c r="DD37">
+        <v>1</v>
+      </c>
+      <c r="DE37">
+        <v>1061.3463999999999</v>
+      </c>
+      <c r="DF37">
+        <v>2267.5484000000001</v>
+      </c>
+      <c r="DG37">
+        <v>187</v>
+      </c>
+      <c r="DH37">
+        <v>19.970700000000001</v>
+      </c>
+      <c r="DI37">
+        <v>7.6412000000000004</v>
+      </c>
+      <c r="DJ37">
+        <v>2.1453000000000002</v>
+      </c>
+      <c r="DK37">
+        <v>11.693300000000001</v>
+      </c>
+      <c r="DL37">
+        <v>21.636199999999999</v>
+      </c>
+      <c r="DM37">
+        <v>14.2265</v>
+      </c>
+      <c r="DN37">
+        <v>11.326599999999999</v>
+      </c>
+      <c r="DO37">
+        <v>52.810600000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>42736</v>
+      </c>
+      <c r="B38" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" t="s">
+        <v>130</v>
+      </c>
+      <c r="E38" t="s">
+        <v>131</v>
+      </c>
+      <c r="G38" t="s">
+        <v>132</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>4670</v>
+      </c>
+      <c r="J38">
+        <v>3020</v>
+      </c>
+      <c r="K38">
+        <v>9590</v>
+      </c>
+      <c r="L38" t="s">
+        <v>131</v>
+      </c>
+      <c r="M38" t="s">
+        <v>163</v>
+      </c>
+      <c r="N38" t="s">
+        <v>133</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
+        <v>600</v>
+      </c>
+      <c r="Q38">
+        <v>0</v>
+      </c>
+      <c r="R38">
+        <v>6871</v>
+      </c>
+      <c r="S38">
+        <v>1</v>
+      </c>
+      <c r="T38">
+        <v>1</v>
+      </c>
+      <c r="U38">
+        <v>1</v>
+      </c>
+      <c r="V38">
+        <v>0</v>
+      </c>
+      <c r="W38">
+        <v>1</v>
+      </c>
+      <c r="X38">
+        <v>1</v>
+      </c>
+      <c r="Z38">
+        <v>4.83</v>
+      </c>
+      <c r="AA38">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AB38">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AC38">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD38">
+        <v>1</v>
+      </c>
+      <c r="AE38">
+        <v>1</v>
+      </c>
+      <c r="AF38">
+        <v>0</v>
+      </c>
+      <c r="AG38" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI38" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ38">
+        <v>1.35</v>
+      </c>
+      <c r="AK38">
+        <v>0.73</v>
+      </c>
+      <c r="AN38" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO38" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP38" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ38" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR38" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS38" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT38" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AV38">
+        <v>5.8</v>
+      </c>
+      <c r="BE38">
+        <v>1560.3554999999999</v>
+      </c>
+      <c r="BF38">
+        <v>25.835999999999999</v>
+      </c>
+      <c r="BG38">
+        <v>59.607999999999997</v>
+      </c>
+      <c r="BH38">
+        <v>1.01E-2</v>
+      </c>
+      <c r="BI38">
+        <v>9764.7281000000003</v>
+      </c>
+      <c r="BJ38">
+        <v>163.8159</v>
+      </c>
+      <c r="BK38">
+        <v>9764.7281000000003</v>
+      </c>
+      <c r="BL38">
+        <v>163.8159</v>
+      </c>
+      <c r="BM38">
+        <v>9764.7281000000003</v>
+      </c>
+      <c r="BN38">
+        <v>163.8159</v>
+      </c>
+      <c r="BO38">
+        <v>9764.7281000000003</v>
+      </c>
+      <c r="BP38">
+        <v>163.8159</v>
+      </c>
+      <c r="BQ38">
+        <v>9764.7281000000003</v>
+      </c>
+      <c r="BR38">
+        <v>163.8159</v>
+      </c>
+      <c r="BS38" s="10">
+        <v>19.595199999999998</v>
+      </c>
+      <c r="BT38">
+        <v>6.4885000000000002</v>
+      </c>
+      <c r="BV38">
+        <v>512.74360000000001</v>
+      </c>
+      <c r="BW38">
+        <v>169.78270000000001</v>
+      </c>
+      <c r="BY38">
+        <v>40.379899999999999</v>
+      </c>
+      <c r="BZ38">
+        <v>45.504899999999999</v>
+      </c>
+      <c r="CA38">
+        <v>19.723299999999998</v>
+      </c>
+      <c r="CB38">
+        <v>0.83030000000000004</v>
+      </c>
+      <c r="CC38">
+        <v>0</v>
+      </c>
+      <c r="CD38">
+        <v>0</v>
+      </c>
+      <c r="CE38">
+        <v>1.5343</v>
+      </c>
+      <c r="CI38">
+        <v>1.5343</v>
+      </c>
+      <c r="CJ38">
+        <v>0</v>
+      </c>
+      <c r="CK38">
+        <v>7.8399999999999997E-2</v>
+      </c>
+      <c r="CL38">
+        <v>3.61E-2</v>
+      </c>
+      <c r="CM38">
+        <v>0.41870000000000002</v>
+      </c>
+      <c r="CN38">
+        <v>0</v>
+      </c>
+      <c r="CO38">
+        <v>0</v>
+      </c>
+      <c r="CP38">
+        <v>0.37930000000000003</v>
+      </c>
+      <c r="CQ38">
+        <v>1.9198999999999999</v>
+      </c>
+      <c r="CR38">
+        <v>0</v>
+      </c>
+      <c r="CS38">
+        <v>9.6324000000000005</v>
+      </c>
+      <c r="CT38">
+        <v>4.9301000000000004</v>
+      </c>
+      <c r="CU38">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+      <c r="CV38">
+        <v>0</v>
+      </c>
+      <c r="CW38">
+        <v>0.6</v>
+      </c>
+      <c r="CX38">
+        <v>-0.63390000000000002</v>
+      </c>
+      <c r="CY38">
+        <v>11.062799999999999</v>
+      </c>
+      <c r="CZ38">
+        <v>10.257199999999999</v>
+      </c>
+      <c r="DA38">
+        <v>71.373999999999995</v>
+      </c>
+      <c r="DB38">
+        <v>85</v>
+      </c>
+      <c r="DC38">
+        <v>1</v>
+      </c>
+      <c r="DD38">
+        <v>1</v>
+      </c>
+      <c r="DE38">
+        <v>1667.6945000000001</v>
+      </c>
+      <c r="DF38">
+        <v>2267.5484000000001</v>
+      </c>
+      <c r="DG38">
+        <v>41</v>
+      </c>
+      <c r="DH38">
+        <v>7.306</v>
+      </c>
+      <c r="DI38">
+        <v>6.0247000000000002</v>
+      </c>
+      <c r="DJ38">
+        <v>3.8540000000000001</v>
+      </c>
+      <c r="DK38">
+        <v>7.1999000000000004</v>
+      </c>
+      <c r="DL38">
+        <v>8.3960000000000008</v>
+      </c>
+      <c r="DM38">
+        <v>4.1444000000000001</v>
+      </c>
+      <c r="DN38">
+        <v>3.6652</v>
+      </c>
+      <c r="DO38">
+        <v>83.794399999999996</v>
+      </c>
+    </row>
+    <row r="39" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" t="s">
+        <v>179</v>
+      </c>
+      <c r="C39" t="s">
+        <v>143</v>
+      </c>
+      <c r="D39" t="s">
+        <v>130</v>
+      </c>
+      <c r="E39" t="s">
+        <v>131</v>
+      </c>
+      <c r="G39" t="s">
+        <v>132</v>
+      </c>
+      <c r="H39">
+        <v>0</v>
+      </c>
+      <c r="I39">
+        <v>4670</v>
+      </c>
+      <c r="J39">
+        <v>3020</v>
+      </c>
+      <c r="K39">
+        <v>9590</v>
+      </c>
+      <c r="L39" t="s">
+        <v>131</v>
+      </c>
+      <c r="M39" t="s">
+        <v>163</v>
+      </c>
+      <c r="N39" t="s">
+        <v>133</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <v>600</v>
+      </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>6871</v>
+      </c>
+      <c r="S39">
+        <v>1</v>
+      </c>
+      <c r="T39">
+        <v>1</v>
+      </c>
+      <c r="U39">
+        <v>1</v>
+      </c>
+      <c r="V39">
+        <v>0</v>
+      </c>
+      <c r="W39">
+        <v>1</v>
+      </c>
+      <c r="X39">
+        <v>1</v>
+      </c>
+      <c r="Z39">
+        <v>4.83</v>
+      </c>
+      <c r="AA39">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AB39">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AC39">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD39">
+        <v>1</v>
+      </c>
+      <c r="AE39">
+        <v>1</v>
+      </c>
+      <c r="AF39">
+        <v>0</v>
+      </c>
+      <c r="AG39" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH39" t="s">
+        <v>180</v>
+      </c>
+      <c r="AI39" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ39">
+        <v>3.4</v>
+      </c>
+      <c r="AK39">
+        <v>0.62</v>
+      </c>
+      <c r="AN39" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO39" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP39" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ39" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR39" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS39" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT39" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU39" t="s">
+        <v>180</v>
+      </c>
+      <c r="AV39">
+        <v>6.2</v>
+      </c>
+      <c r="BE39">
+        <v>1563.3505</v>
+      </c>
+      <c r="BF39">
+        <v>25.835999999999999</v>
+      </c>
+      <c r="BG39">
+        <v>59.4938</v>
+      </c>
+      <c r="BH39">
+        <v>1.01E-2</v>
+      </c>
+      <c r="BI39">
+        <v>9500.7245999999996</v>
+      </c>
+      <c r="BJ39">
+        <v>159.69280000000001</v>
+      </c>
+      <c r="BK39">
+        <v>9500.7245999999996</v>
+      </c>
+      <c r="BL39">
+        <v>159.69280000000001</v>
+      </c>
+      <c r="BM39">
+        <v>9500.7245999999996</v>
+      </c>
+      <c r="BN39">
+        <v>159.69280000000001</v>
+      </c>
+      <c r="BO39">
+        <v>9500.7245999999996</v>
+      </c>
+      <c r="BP39">
+        <v>159.69280000000001</v>
+      </c>
+      <c r="BQ39">
+        <v>9500.7245999999996</v>
+      </c>
+      <c r="BR39">
+        <v>159.69280000000001</v>
+      </c>
+      <c r="BS39" s="10">
+        <v>19.102</v>
+      </c>
+      <c r="BT39">
+        <v>6.3251999999999997</v>
+      </c>
+      <c r="BV39">
+        <v>499.83839999999998</v>
+      </c>
+      <c r="BW39">
+        <v>165.5094</v>
+      </c>
+      <c r="BY39">
+        <v>40.28</v>
+      </c>
+      <c r="BZ39">
+        <v>45.100999999999999</v>
+      </c>
+      <c r="CA39">
+        <v>19.585699999999999</v>
+      </c>
+      <c r="CB39">
+        <v>0.71830000000000005</v>
+      </c>
+      <c r="CC39">
+        <v>0</v>
+      </c>
+      <c r="CD39">
+        <v>0</v>
+      </c>
+      <c r="CE39">
+        <v>1.5373000000000001</v>
+      </c>
+      <c r="CI39">
+        <v>1.5373000000000001</v>
+      </c>
+      <c r="CJ39">
+        <v>0</v>
+      </c>
+      <c r="CK39">
+        <v>5.3E-3</v>
+      </c>
+      <c r="CL39">
+        <v>5.9799999999999999E-2</v>
+      </c>
+      <c r="CM39">
+        <v>0.44409999999999999</v>
+      </c>
+      <c r="CN39">
+        <v>0</v>
+      </c>
+      <c r="CO39">
+        <v>0</v>
+      </c>
+      <c r="CP39">
+        <v>0.3765</v>
+      </c>
+      <c r="CQ39">
+        <v>1.9541999999999999</v>
+      </c>
+      <c r="CR39">
+        <v>0</v>
+      </c>
+      <c r="CS39">
+        <v>9.6201000000000008</v>
+      </c>
+      <c r="CT39">
+        <v>4.9301000000000004</v>
+      </c>
+      <c r="CU39">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+      <c r="CV39">
+        <v>0</v>
+      </c>
+      <c r="CW39">
+        <v>0.54179999999999995</v>
+      </c>
+      <c r="CX39">
+        <v>-0.65390000000000004</v>
+      </c>
+      <c r="CY39">
+        <v>12.016299999999999</v>
+      </c>
+      <c r="CZ39">
+        <v>9.7856000000000005</v>
+      </c>
+      <c r="DA39">
+        <v>70.906099999999995</v>
+      </c>
+      <c r="DB39">
+        <v>85</v>
+      </c>
+      <c r="DC39">
+        <v>1</v>
+      </c>
+      <c r="DD39">
+        <v>1</v>
+      </c>
+      <c r="DE39">
+        <v>1529.8036999999999</v>
+      </c>
+      <c r="DF39">
+        <v>2058.6812</v>
+      </c>
+      <c r="DG39">
+        <v>71</v>
+      </c>
+      <c r="DH39">
+        <v>7.2919999999999998</v>
+      </c>
+      <c r="DI39">
+        <v>7.1409000000000002</v>
+      </c>
+      <c r="DJ39">
+        <v>3.5097</v>
+      </c>
+      <c r="DK39">
+        <v>7.1957000000000004</v>
+      </c>
+      <c r="DL39">
+        <v>7.9516999999999998</v>
+      </c>
+      <c r="DM39">
+        <v>1.2159</v>
+      </c>
+      <c r="DN39">
+        <v>0.53200000000000003</v>
+      </c>
+      <c r="DO39">
+        <v>2.4116</v>
+      </c>
+      <c r="DP39">
+        <v>3.8666999999999998</v>
+      </c>
+      <c r="DQ39">
+        <v>3.0802</v>
+      </c>
+      <c r="DR39">
+        <v>80.942099999999996</v>
+      </c>
+    </row>
+    <row r="40" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>42737</v>
+      </c>
+      <c r="B40" t="s">
+        <v>179</v>
+      </c>
+      <c r="C40" t="s">
+        <v>144</v>
+      </c>
+      <c r="D40" t="s">
+        <v>130</v>
+      </c>
+      <c r="E40" t="s">
+        <v>131</v>
+      </c>
+      <c r="G40" t="s">
+        <v>132</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>4670</v>
+      </c>
+      <c r="J40">
+        <v>3020</v>
+      </c>
+      <c r="K40">
+        <v>9590</v>
+      </c>
+      <c r="L40" t="s">
+        <v>131</v>
+      </c>
+      <c r="M40" t="s">
+        <v>163</v>
+      </c>
+      <c r="N40" t="s">
+        <v>133</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
+        <v>600</v>
+      </c>
+      <c r="Q40">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>6871</v>
+      </c>
+      <c r="S40">
+        <v>1</v>
+      </c>
+      <c r="T40">
+        <v>1</v>
+      </c>
+      <c r="U40">
+        <v>1</v>
+      </c>
+      <c r="V40">
+        <v>0</v>
+      </c>
+      <c r="W40">
+        <v>1</v>
+      </c>
+      <c r="X40">
+        <v>1</v>
+      </c>
+      <c r="Z40">
+        <v>4.83</v>
+      </c>
+      <c r="AA40">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AB40">
+        <v>7.30621220357534E-3</v>
+      </c>
+      <c r="AC40">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD40">
+        <v>1</v>
+      </c>
+      <c r="AE40">
+        <v>1</v>
+      </c>
+      <c r="AF40">
+        <v>0</v>
+      </c>
+      <c r="AG40" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH40" t="s">
+        <v>180</v>
+      </c>
+      <c r="AI40" t="s">
+        <v>181</v>
+      </c>
+      <c r="AJ40">
+        <v>3.4</v>
+      </c>
+      <c r="AK40">
+        <v>0.62</v>
+      </c>
+      <c r="AN40" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO40" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP40" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ40" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR40" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS40" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT40" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU40" t="s">
+        <v>180</v>
+      </c>
+      <c r="AV40">
+        <v>6.2</v>
+      </c>
+      <c r="BE40">
+        <v>3211.7003</v>
+      </c>
+      <c r="BF40">
+        <v>27.815999999999999</v>
+      </c>
+      <c r="BG40">
+        <v>31.178999999999998</v>
+      </c>
+      <c r="BH40">
+        <v>-1.5800000000000002E-2</v>
+      </c>
+      <c r="BI40">
+        <v>5507.6671999999999</v>
+      </c>
+      <c r="BJ40">
+        <v>176.64670000000001</v>
+      </c>
+      <c r="BK40">
+        <v>5507.6671999999999</v>
+      </c>
+      <c r="BL40">
+        <v>176.64670000000001</v>
+      </c>
+      <c r="BM40">
+        <v>5507.6671999999999</v>
+      </c>
+      <c r="BN40">
+        <v>176.64670000000001</v>
+      </c>
+      <c r="BO40">
+        <v>5507.6671999999999</v>
+      </c>
+      <c r="BP40">
+        <v>176.64670000000001</v>
+      </c>
+      <c r="BQ40">
+        <v>5507.6671999999999</v>
+      </c>
+      <c r="BR40">
+        <v>176.64670000000001</v>
+      </c>
+      <c r="BS40" s="2">
+        <v>21.13</v>
+      </c>
+      <c r="BT40">
+        <v>6.9966999999999997</v>
+      </c>
+      <c r="BV40">
+        <v>552.90419999999995</v>
+      </c>
+      <c r="BW40">
+        <v>183.08080000000001</v>
+      </c>
+      <c r="BY40">
+        <v>21.0442</v>
+      </c>
+      <c r="BZ40">
+        <v>25.247199999999999</v>
+      </c>
+      <c r="CA40">
+        <v>22.524000000000001</v>
+      </c>
+      <c r="CB40">
+        <v>1.0708</v>
+      </c>
+      <c r="CC40">
+        <v>0</v>
+      </c>
+      <c r="CD40">
+        <v>0</v>
+      </c>
+      <c r="CE40">
+        <v>3.1581999999999999</v>
+      </c>
+      <c r="CI40">
+        <v>3.1581999999999999</v>
+      </c>
+      <c r="CJ40">
+        <v>0</v>
+      </c>
+      <c r="CK40">
+        <v>2.87E-2</v>
+      </c>
+      <c r="CL40">
+        <v>0.26429999999999998</v>
+      </c>
+      <c r="CM40">
+        <v>0.69120000000000004</v>
+      </c>
+      <c r="CN40">
+        <v>0</v>
+      </c>
+      <c r="CO40">
+        <v>0</v>
+      </c>
+      <c r="CP40">
+        <v>0.41589999999999999</v>
+      </c>
+      <c r="CQ40">
+        <v>6.5374999999999996</v>
+      </c>
+      <c r="CR40">
+        <v>0</v>
+      </c>
+      <c r="CS40">
+        <v>5.3140999999999998</v>
+      </c>
+      <c r="CT40">
+        <v>5.3079000000000001</v>
+      </c>
+      <c r="CU40">
+        <v>-1E-4</v>
+      </c>
+      <c r="CV40">
+        <v>0</v>
+      </c>
+      <c r="CW40">
+        <v>0.61509999999999998</v>
+      </c>
+      <c r="CX40">
+        <v>-0.84019999999999995</v>
+      </c>
+      <c r="CY40">
+        <v>17.136900000000001</v>
+      </c>
+      <c r="CZ40">
+        <v>12.6593</v>
+      </c>
+      <c r="DA40">
+        <v>50.307699999999997</v>
+      </c>
+      <c r="DB40">
+        <v>85</v>
+      </c>
+      <c r="DC40">
+        <v>1</v>
+      </c>
+      <c r="DD40">
+        <v>1</v>
+      </c>
+      <c r="DE40">
+        <v>1011.0384</v>
+      </c>
+      <c r="DF40">
+        <v>2058.6812</v>
+      </c>
+      <c r="DG40">
+        <v>315</v>
+      </c>
+      <c r="DH40">
+        <v>19.896000000000001</v>
+      </c>
+      <c r="DI40">
+        <v>10.099500000000001</v>
+      </c>
+      <c r="DJ40">
+        <v>2.1766999999999999</v>
+      </c>
+      <c r="DK40">
+        <v>11.595700000000001</v>
+      </c>
+      <c r="DL40">
+        <v>21.4802</v>
+      </c>
+      <c r="DM40">
+        <v>3.3336999999999999</v>
+      </c>
+      <c r="DN40">
+        <v>3.8067000000000002</v>
+      </c>
+      <c r="DO40">
+        <v>4.5907999999999998</v>
+      </c>
+      <c r="DP40">
+        <v>12.8131</v>
+      </c>
+      <c r="DQ40">
+        <v>5.9470000000000001</v>
+      </c>
+      <c r="DR40">
+        <v>48.028399999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>190</v>
+      </c>
+      <c r="B41" t="s">
+        <v>161</v>
+      </c>
+      <c r="C41" t="s">
+        <v>162</v>
+      </c>
+      <c r="D41" t="s">
+        <v>130</v>
+      </c>
+      <c r="E41" t="s">
+        <v>131</v>
+      </c>
+      <c r="G41" t="s">
+        <v>132</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>4670</v>
+      </c>
+      <c r="J41">
+        <v>3020</v>
+      </c>
+      <c r="K41">
+        <v>9590</v>
+      </c>
+      <c r="L41" t="s">
+        <v>131</v>
+      </c>
+      <c r="M41" t="s">
+        <v>163</v>
+      </c>
+      <c r="N41" t="s">
+        <v>133</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>600</v>
+      </c>
+      <c r="Q41">
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>6871</v>
+      </c>
+      <c r="S41">
+        <v>1</v>
+      </c>
+      <c r="T41">
+        <v>1</v>
+      </c>
+      <c r="U41">
+        <v>1</v>
+      </c>
+      <c r="V41">
+        <v>0</v>
+      </c>
+      <c r="W41">
+        <v>1</v>
+      </c>
+      <c r="X41">
+        <v>1</v>
+      </c>
+      <c r="Z41">
+        <v>4.83</v>
+      </c>
+      <c r="AA41">
+        <v>6.7632194436728502E-3</v>
+      </c>
+      <c r="AB41">
+        <v>6.7632194436728502E-3</v>
+      </c>
+      <c r="AC41">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD41">
+        <v>1</v>
+      </c>
+      <c r="AE41">
+        <v>3</v>
+      </c>
+      <c r="AF41">
+        <v>0</v>
+      </c>
+      <c r="AG41" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH41" t="s">
+        <v>164</v>
+      </c>
+      <c r="AI41" t="s">
+        <v>135</v>
+      </c>
+      <c r="AJ41">
+        <v>6.7</v>
+      </c>
+      <c r="AK41">
+        <v>0.73</v>
+      </c>
+      <c r="AL41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP41" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS41" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT41" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU41" t="s">
+        <v>164</v>
+      </c>
+      <c r="AV41">
+        <v>4.18</v>
+      </c>
+      <c r="BE41">
+        <v>1570.0481</v>
+      </c>
+      <c r="BF41">
+        <v>25.835999999999999</v>
+      </c>
+      <c r="BG41">
+        <v>59.24</v>
+      </c>
+      <c r="BH41">
+        <v>1.01E-2</v>
+      </c>
+      <c r="BI41">
+        <v>10285.6561</v>
+      </c>
+      <c r="BJ41">
+        <v>173.62700000000001</v>
+      </c>
+      <c r="BK41">
+        <v>10285.6561</v>
+      </c>
+      <c r="BL41">
+        <v>173.62700000000001</v>
+      </c>
+      <c r="BM41">
+        <v>10285.6561</v>
+      </c>
+      <c r="BN41">
+        <v>173.62700000000001</v>
+      </c>
+      <c r="BO41">
+        <v>10285.6561</v>
+      </c>
+      <c r="BP41">
+        <v>173.62700000000001</v>
+      </c>
+      <c r="BQ41">
+        <v>10285.6561</v>
+      </c>
+      <c r="BR41">
+        <v>173.62700000000001</v>
+      </c>
+      <c r="BS41" s="2">
+        <v>20.768799999999999</v>
+      </c>
+      <c r="BT41">
+        <v>6.8771000000000004</v>
+      </c>
+      <c r="BV41">
+        <v>543.45240000000001</v>
+      </c>
+      <c r="BW41">
+        <v>179.9511</v>
+      </c>
+      <c r="BY41">
+        <v>42.134599999999999</v>
+      </c>
+      <c r="BZ41">
+        <v>51.103299999999997</v>
+      </c>
+      <c r="CA41">
+        <v>22.287400000000002</v>
+      </c>
+      <c r="CB41">
+        <v>0.74780000000000002</v>
+      </c>
+      <c r="CC41">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="CD41">
+        <v>0</v>
+      </c>
+      <c r="CE41">
+        <v>1.5439000000000001</v>
+      </c>
+      <c r="CI41">
+        <v>1.5439000000000001</v>
+      </c>
+      <c r="CJ41">
+        <v>2.29E-2</v>
+      </c>
+      <c r="CK41">
+        <v>0</v>
+      </c>
+      <c r="CL41">
+        <v>0</v>
+      </c>
+      <c r="CM41">
+        <v>1.7982</v>
+      </c>
+      <c r="CN41">
+        <v>0</v>
+      </c>
+      <c r="CO41">
+        <v>0</v>
+      </c>
+      <c r="CP41">
+        <v>0.89180000000000004</v>
+      </c>
+      <c r="CQ41">
+        <v>1.8145</v>
+      </c>
+      <c r="CR41">
+        <v>0</v>
+      </c>
+      <c r="CS41">
+        <v>10.904199999999999</v>
+      </c>
+      <c r="CT41">
+        <v>4.5636999999999999</v>
+      </c>
+      <c r="CU41">
+        <v>-2.0000000000000001E-4</v>
+      </c>
+      <c r="CV41">
+        <v>0</v>
+      </c>
+      <c r="CW41">
+        <v>0.67849999999999999</v>
+      </c>
+      <c r="CX41">
+        <v>-0.59219999999999995</v>
+      </c>
+      <c r="CY41">
+        <v>11.315899999999999</v>
+      </c>
+      <c r="CZ41">
+        <v>12.3415</v>
+      </c>
+      <c r="DA41">
+        <v>69.081599999999995</v>
+      </c>
+      <c r="DB41">
+        <v>85</v>
+      </c>
+      <c r="DC41">
+        <v>1</v>
+      </c>
+      <c r="DD41">
+        <v>1</v>
+      </c>
+      <c r="DE41">
+        <v>1453.1723999999999</v>
+      </c>
+      <c r="DF41">
+        <v>2328.2910000000002</v>
+      </c>
+      <c r="DG41">
+        <v>55</v>
+      </c>
+      <c r="DH41">
+        <v>7.2609000000000004</v>
+      </c>
+      <c r="DI41">
+        <v>5.1551</v>
+      </c>
+      <c r="DJ41">
+        <v>3.1116999999999999</v>
+      </c>
+      <c r="DK41">
+        <v>7.2786999999999997</v>
+      </c>
+      <c r="DL41">
+        <v>12.426</v>
+      </c>
+      <c r="DM41">
+        <v>0.1822</v>
+      </c>
+      <c r="DN41">
+        <v>2.8713000000000002</v>
+      </c>
+      <c r="DO41">
+        <v>4.4143999999999997</v>
+      </c>
+      <c r="DP41">
+        <v>9.8996999999999993</v>
+      </c>
+      <c r="DQ41">
+        <v>17.389600000000002</v>
+      </c>
+      <c r="DR41">
+        <v>52.816800000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>42738</v>
+      </c>
+      <c r="B42" t="s">
+        <v>161</v>
+      </c>
+      <c r="C42" t="s">
+        <v>165</v>
+      </c>
+      <c r="D42" t="s">
+        <v>130</v>
+      </c>
+      <c r="E42" t="s">
+        <v>131</v>
+      </c>
+      <c r="G42" t="s">
+        <v>132</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>4670</v>
+      </c>
+      <c r="J42">
+        <v>3020</v>
+      </c>
+      <c r="K42">
+        <v>9590</v>
+      </c>
+      <c r="L42" t="s">
+        <v>131</v>
+      </c>
+      <c r="M42" t="s">
+        <v>163</v>
+      </c>
+      <c r="N42" t="s">
+        <v>133</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42">
+        <v>600</v>
+      </c>
+      <c r="Q42">
+        <v>0</v>
+      </c>
+      <c r="R42">
+        <v>6871</v>
+      </c>
+      <c r="S42">
+        <v>1</v>
+      </c>
+      <c r="T42">
+        <v>1</v>
+      </c>
+      <c r="U42">
+        <v>1</v>
+      </c>
+      <c r="V42">
+        <v>0</v>
+      </c>
+      <c r="W42">
+        <v>1</v>
+      </c>
+      <c r="X42">
+        <v>1</v>
+      </c>
+      <c r="Z42">
+        <v>4.83</v>
+      </c>
+      <c r="AA42">
+        <v>6.7632194436728502E-3</v>
+      </c>
+      <c r="AB42">
+        <v>6.7632194436728502E-3</v>
+      </c>
+      <c r="AC42">
+        <v>0.42099999999999999</v>
+      </c>
+      <c r="AD42">
+        <v>1</v>
+      </c>
+      <c r="AE42">
+        <v>3</v>
+      </c>
+      <c r="AF42">
+        <v>0</v>
+      </c>
+      <c r="AG42" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH42" t="s">
+        <v>164</v>
+      </c>
+      <c r="AI42" t="s">
+        <v>135</v>
+      </c>
+      <c r="AJ42">
+        <v>6.7</v>
+      </c>
+      <c r="AK42">
+        <v>0.73</v>
+      </c>
+      <c r="AL42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP42" t="s">
+        <v>137</v>
+      </c>
+      <c r="AQ42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS42" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT42" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU42" t="s">
+        <v>164</v>
+      </c>
+      <c r="AV42">
+        <v>4.18</v>
+      </c>
+      <c r="BE42">
+        <v>3235.4205999999999</v>
+      </c>
+      <c r="BF42">
+        <v>27.815999999999999</v>
+      </c>
+      <c r="BG42">
+        <v>30.950399999999998</v>
+      </c>
+      <c r="BH42">
+        <v>-1.5800000000000002E-2</v>
+      </c>
+      <c r="BI42">
+        <v>5973.3266999999996</v>
+      </c>
+      <c r="BJ42">
+        <v>192.9967</v>
+      </c>
+      <c r="BK42">
+        <v>5973.3266999999996</v>
+      </c>
+      <c r="BL42">
+        <v>192.9967</v>
+      </c>
+      <c r="BM42">
+        <v>5973.3266999999996</v>
+      </c>
+      <c r="BN42">
+        <v>192.9967</v>
+      </c>
+      <c r="BO42">
+        <v>5973.3266999999996</v>
+      </c>
+      <c r="BP42">
+        <v>192.9967</v>
+      </c>
+      <c r="BQ42">
+        <v>5973.3266999999996</v>
+      </c>
+      <c r="BR42">
+        <v>192.9967</v>
+      </c>
+      <c r="BS42" s="10">
+        <v>23.085699999999999</v>
+      </c>
+      <c r="BT42">
+        <v>7.6443000000000003</v>
+      </c>
+      <c r="BV42">
+        <v>604.07960000000003</v>
+      </c>
+      <c r="BW42">
+        <v>200.0264</v>
+      </c>
+      <c r="BY42">
+        <v>21.456600000000002</v>
+      </c>
+      <c r="BZ42">
+        <v>28.352499999999999</v>
+      </c>
+      <c r="CA42">
+        <v>25.481100000000001</v>
+      </c>
+      <c r="CB42">
+        <v>1.6879</v>
+      </c>
+      <c r="CC42">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="CD42">
+        <v>0</v>
+      </c>
+      <c r="CE42">
+        <v>3.1815000000000002</v>
+      </c>
+      <c r="CI42">
+        <v>3.1815000000000002</v>
+      </c>
+      <c r="CJ42">
+        <v>0.12770000000000001</v>
+      </c>
+      <c r="CK42">
+        <v>0</v>
+      </c>
+      <c r="CL42">
+        <v>0</v>
+      </c>
+      <c r="CM42">
+        <v>2.3860000000000001</v>
+      </c>
+      <c r="CN42">
+        <v>0</v>
+      </c>
+      <c r="CO42">
+        <v>0</v>
+      </c>
+      <c r="CP42">
+        <v>0.92230000000000001</v>
+      </c>
+      <c r="CQ42">
+        <v>6.0845000000000002</v>
+      </c>
+      <c r="CR42">
+        <v>0</v>
+      </c>
+      <c r="CS42">
+        <v>6.1776</v>
+      </c>
+      <c r="CT42">
+        <v>4.9134000000000002</v>
+      </c>
+      <c r="CU42">
+        <v>-1E-4</v>
+      </c>
+      <c r="CV42">
+        <v>0</v>
+      </c>
+      <c r="CW42">
+        <v>0.77039999999999997</v>
+      </c>
+      <c r="CX42">
+        <v>-0.71389999999999998</v>
+      </c>
+      <c r="CY42">
+        <v>15.3523</v>
+      </c>
+      <c r="CZ42">
+        <v>15.9184</v>
+      </c>
+      <c r="DA42">
+        <v>48.979100000000003</v>
+      </c>
+      <c r="DB42">
+        <v>85</v>
+      </c>
+      <c r="DC42">
+        <v>1</v>
+      </c>
+      <c r="DD42">
+        <v>1</v>
+      </c>
+      <c r="DE42">
+        <v>1255.9588000000001</v>
+      </c>
+      <c r="DF42">
+        <v>2311.0162999999998</v>
+      </c>
+      <c r="DG42">
+        <v>200</v>
+      </c>
+      <c r="DH42">
+        <v>19.7501</v>
+      </c>
+      <c r="DI42">
+        <v>2.5137999999999998</v>
+      </c>
+      <c r="DJ42">
+        <v>2.1617000000000002</v>
+      </c>
+      <c r="DK42">
+        <v>11.484400000000001</v>
+      </c>
+      <c r="DL42">
+        <v>28.363800000000001</v>
+      </c>
+      <c r="DM42">
+        <v>0.26540000000000002</v>
+      </c>
+      <c r="DN42">
+        <v>7.2965</v>
+      </c>
+      <c r="DO42">
+        <v>16.077400000000001</v>
+      </c>
+      <c r="DP42">
+        <v>14.389699999999999</v>
+      </c>
+      <c r="DQ42">
+        <v>25.304099999999998</v>
+      </c>
+      <c r="DR42">
+        <v>8.3031000000000006</v>
+      </c>
+    </row>
+    <row r="43" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>160</v>
+      </c>
+      <c r="B43" t="s">
+        <v>167</v>
+      </c>
+      <c r="C43" t="s">
+        <v>168</v>
+      </c>
+      <c r="D43" t="s">
+        <v>130</v>
+      </c>
+      <c r="E43" t="s">
+        <v>131</v>
+      </c>
+      <c r="G43" t="s">
+        <v>132</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>8229</v>
+      </c>
+      <c r="J43">
+        <v>19300</v>
+      </c>
+      <c r="K43">
+        <v>35029</v>
+      </c>
+      <c r="L43" t="s">
+        <v>131</v>
+      </c>
+      <c r="M43" t="s">
+        <v>169</v>
+      </c>
+      <c r="N43" t="s">
+        <v>133</v>
+      </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>600</v>
+      </c>
+      <c r="Q43">
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>12740</v>
+      </c>
+      <c r="S43">
+        <v>1</v>
+      </c>
+      <c r="T43">
+        <v>1</v>
+      </c>
+      <c r="U43">
+        <v>1</v>
+      </c>
+      <c r="V43">
+        <v>0</v>
+      </c>
+      <c r="W43">
+        <v>1</v>
+      </c>
+      <c r="X43">
+        <v>1</v>
+      </c>
+      <c r="Z43">
+        <v>5.3</v>
+      </c>
+      <c r="AA43">
+        <v>5.9060053756203601E-3</v>
+      </c>
+      <c r="AB43">
+        <v>5.9060053756203601E-3</v>
+      </c>
+      <c r="AC43">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="AD43">
+        <v>1</v>
+      </c>
+      <c r="AE43">
+        <v>4</v>
+      </c>
+      <c r="AF43">
+        <v>0</v>
+      </c>
+      <c r="AG43" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH43" t="s">
+        <v>147</v>
+      </c>
+      <c r="AI43" t="s">
+        <v>148</v>
+      </c>
+      <c r="AJ43">
+        <v>14.93</v>
+      </c>
+      <c r="AK43">
+        <v>1</v>
+      </c>
+      <c r="AL43" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM43" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN43" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO43" t="s">
+        <v>132</v>
+      </c>
+      <c r="AP43" t="s">
+        <v>149</v>
+      </c>
+      <c r="AQ43" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR43" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS43" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT43" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU43" t="s">
+        <v>147</v>
+      </c>
+      <c r="AV43">
+        <v>2.64</v>
+      </c>
+      <c r="BE43">
+        <v>5364.7655999999997</v>
+      </c>
+      <c r="BF43">
+        <v>108.191</v>
+      </c>
+      <c r="BG43">
+        <v>72.600999999999999</v>
+      </c>
+      <c r="BH43">
+        <v>0.17019999999999999</v>
+      </c>
+      <c r="BI43">
+        <v>22400.1132</v>
+      </c>
+      <c r="BJ43">
+        <v>308.53710000000001</v>
+      </c>
+      <c r="BK43">
+        <v>22400.1132</v>
+      </c>
+      <c r="BL43">
+        <v>308.53710000000001</v>
+      </c>
+      <c r="BM43">
+        <v>22400.1132</v>
+      </c>
+      <c r="BN43">
+        <v>308.53710000000001</v>
+      </c>
+      <c r="BO43">
+        <v>22400.1132</v>
+      </c>
+      <c r="BP43">
+        <v>308.53710000000001</v>
+      </c>
+      <c r="BQ43">
+        <v>22400.1132</v>
+      </c>
+      <c r="BR43">
+        <v>308.53710000000001</v>
+      </c>
+      <c r="BS43" s="2">
+        <v>36.906300000000002</v>
+      </c>
+      <c r="BT43">
+        <v>1.9121999999999999</v>
+      </c>
+      <c r="BV43">
+        <v>965.721</v>
+      </c>
+      <c r="BW43">
+        <v>50.037399999999998</v>
+      </c>
+      <c r="BY43">
+        <v>100.17959999999999</v>
+      </c>
+      <c r="BZ43">
+        <v>116.4485</v>
+      </c>
+      <c r="CA43">
+        <v>173.53299999999999</v>
+      </c>
+      <c r="CB43">
+        <v>5.4751000000000003</v>
+      </c>
+      <c r="CC43">
+        <v>0</v>
+      </c>
+      <c r="CD43">
+        <v>0</v>
+      </c>
+      <c r="CE43">
+        <v>7.4511000000000003</v>
+      </c>
+      <c r="CH43">
+        <v>3.9925999999999999</v>
+      </c>
+      <c r="CI43">
+        <v>11.4437</v>
+      </c>
+      <c r="CJ43">
+        <v>4.9799999999999997E-2</v>
+      </c>
+      <c r="CK43">
+        <v>0</v>
+      </c>
+      <c r="CL43">
+        <v>0</v>
+      </c>
+      <c r="CM43">
+        <v>8.4329000000000001</v>
+      </c>
+      <c r="CN43">
+        <v>2.0390999999999999</v>
+      </c>
+      <c r="CO43">
+        <v>0</v>
+      </c>
+      <c r="CP43">
+        <v>7.5175999999999998</v>
+      </c>
+      <c r="CQ43">
+        <v>23.3383</v>
+      </c>
+      <c r="CR43">
+        <v>0</v>
+      </c>
+      <c r="CS43">
+        <v>54.272799999999997</v>
+      </c>
+      <c r="CT43">
+        <v>60.961199999999998</v>
+      </c>
+      <c r="CU43">
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="CV43">
+        <v>0</v>
+      </c>
+      <c r="CW43">
+        <v>0.38229999999999997</v>
+      </c>
+      <c r="CX43">
+        <v>-0.48130000000000001</v>
+      </c>
+      <c r="CY43">
+        <v>6.6596000000000002</v>
+      </c>
+      <c r="CZ43">
+        <v>4.7657999999999996</v>
+      </c>
+      <c r="DA43">
+        <v>84.026499999999999</v>
+      </c>
+      <c r="DB43">
+        <v>85</v>
+      </c>
+      <c r="DC43">
+        <v>1</v>
+      </c>
+      <c r="DD43">
+        <v>1</v>
+      </c>
+      <c r="DE43">
+        <v>1179.2496000000001</v>
+      </c>
+      <c r="DF43">
+        <v>1774.8970999999999</v>
+      </c>
+      <c r="DG43">
+        <v>95</v>
+      </c>
+      <c r="DH43">
+        <v>4.5481999999999996</v>
+      </c>
+      <c r="DI43">
+        <v>22.119700000000002</v>
+      </c>
+      <c r="DJ43">
+        <v>4.1486000000000001</v>
+      </c>
+      <c r="DK43">
+        <v>2.0455999999999999</v>
+      </c>
+      <c r="DL43">
+        <v>6.2424999999999997</v>
+      </c>
+      <c r="DM43">
+        <v>0</v>
+      </c>
+      <c r="DN43">
+        <v>8.9599999999999999E-2</v>
+      </c>
+      <c r="DO43">
+        <v>0.13439999999999999</v>
+      </c>
+      <c r="DP43">
+        <v>0.20780000000000001</v>
+      </c>
+      <c r="DQ43">
+        <v>0.13120000000000001</v>
+      </c>
+      <c r="DR43">
+        <v>0.27489999999999998</v>
+      </c>
+      <c r="DS43">
+        <v>0.40770000000000001</v>
+      </c>
+      <c r="DT43">
+        <v>0.7984</v>
+      </c>
+      <c r="DU43">
+        <v>5.7752999999999997</v>
+      </c>
+      <c r="DV43">
+        <v>6.7645</v>
+      </c>
+      <c r="DW43">
+        <v>5.9824000000000002</v>
+      </c>
+      <c r="DX43">
+        <v>73.191199999999995</v>
+      </c>
+    </row>
+    <row r="44" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>166</v>
+      </c>
+      <c r="B44" t="s">
+        <v>171</v>
+      </c>
+      <c r="C44" t="s">
+        <v>172</v>
+      </c>
+      <c r="D44" t="s">
+        <v>130</v>
+      </c>
+      <c r="E44" t="s">
+        <v>131</v>
+      </c>
+      <c r="G44" t="s">
+        <v>132</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>9300</v>
+      </c>
+      <c r="J44">
+        <v>7100</v>
+      </c>
+      <c r="K44">
+        <v>18600</v>
+      </c>
+      <c r="L44" t="s">
+        <v>131</v>
+      </c>
+      <c r="M44" t="s">
+        <v>173</v>
+      </c>
+      <c r="N44" t="s">
+        <v>133</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>600</v>
+      </c>
+      <c r="Q44">
+        <v>0</v>
+      </c>
+      <c r="R44">
+        <v>7000</v>
+      </c>
+      <c r="S44">
+        <v>1</v>
+      </c>
+      <c r="T44">
+        <v>1</v>
+      </c>
+      <c r="U44">
+        <v>1</v>
+      </c>
+      <c r="V44">
+        <v>0</v>
+      </c>
+      <c r="W44">
+        <v>1</v>
+      </c>
+      <c r="X44">
+        <v>1</v>
+      </c>
+      <c r="Z44">
+        <v>5.2</v>
+      </c>
+      <c r="AA44">
+        <v>5.6985855186778601E-3</v>
+      </c>
+      <c r="AB44">
+        <v>5.6985855186778601E-3</v>
+      </c>
+      <c r="AC44">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="AD44">
+        <v>1</v>
+      </c>
+      <c r="AE44">
+        <v>2</v>
+      </c>
+      <c r="AF44">
+        <v>0</v>
+      </c>
+      <c r="AG44" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH44" t="s">
+        <v>147</v>
+      </c>
+      <c r="AI44" t="s">
+        <v>148</v>
+      </c>
+      <c r="AJ44">
+        <v>14.93</v>
+      </c>
+      <c r="AK44">
+        <v>1</v>
+      </c>
+      <c r="AL44" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM44" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN44" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO44" t="s">
+        <v>132</v>
+      </c>
+      <c r="AP44" t="s">
+        <v>149</v>
+      </c>
+      <c r="AQ44" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR44" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS44" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT44" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU44" t="s">
+        <v>147</v>
+      </c>
+      <c r="AV44">
+        <v>2.64</v>
+      </c>
+      <c r="BE44">
+        <v>1203.4902</v>
+      </c>
+      <c r="BF44">
+        <v>0.80030000000000001</v>
+      </c>
+      <c r="BG44">
+        <v>2.3940000000000001</v>
+      </c>
+      <c r="BH44">
+        <v>-1.2842</v>
+      </c>
+      <c r="BI44">
+        <v>5825.2356</v>
+      </c>
+      <c r="BJ44">
+        <v>2433.3116</v>
+      </c>
+      <c r="BK44">
+        <v>5825.2356</v>
+      </c>
+      <c r="BL44">
+        <v>2433.3116</v>
+      </c>
+      <c r="BM44">
+        <v>5825.2356</v>
+      </c>
+      <c r="BN44">
+        <v>2433.3116</v>
+      </c>
+      <c r="BO44">
+        <v>5825.2356</v>
+      </c>
+      <c r="BP44">
+        <v>2433.3116</v>
+      </c>
+      <c r="BQ44">
+        <v>5825.2356</v>
+      </c>
+      <c r="BR44">
+        <v>2433.3116</v>
+      </c>
+      <c r="BS44" s="2">
+        <v>291.06599999999997</v>
+      </c>
+      <c r="BT44">
+        <v>40.995199999999997</v>
+      </c>
+      <c r="BV44">
+        <v>7616.2655000000004</v>
+      </c>
+      <c r="BW44">
+        <v>1072.7134000000001</v>
+      </c>
+      <c r="BY44">
+        <v>2.9887000000000001</v>
+      </c>
+      <c r="BZ44">
+        <v>21.9132</v>
+      </c>
+      <c r="CA44">
+        <v>7.3255999999999997</v>
+      </c>
+      <c r="CB44">
+        <v>0.22770000000000001</v>
+      </c>
+      <c r="CC44">
+        <v>-1.4E-3</v>
+      </c>
+      <c r="CD44">
+        <v>1.0028999999999999</v>
+      </c>
+      <c r="CE44">
+        <v>1.1700999999999999</v>
+      </c>
+      <c r="CF44">
+        <v>0.33429999999999999</v>
+      </c>
+      <c r="CG44">
+        <v>3.2865000000000002</v>
+      </c>
+      <c r="CI44">
+        <v>2.173</v>
+      </c>
+      <c r="CJ44">
+        <v>0.2452</v>
+      </c>
+      <c r="CK44">
+        <v>0</v>
+      </c>
+      <c r="CL44">
+        <v>0</v>
+      </c>
+      <c r="CM44">
+        <v>8.8200000000000001E-2</v>
+      </c>
+      <c r="CN44">
+        <v>1.21E-2</v>
+      </c>
+      <c r="CO44">
+        <v>0</v>
+      </c>
+      <c r="CP44">
+        <v>4.8800000000000003E-2</v>
+      </c>
+      <c r="CQ44">
+        <v>0.81069999999999998</v>
+      </c>
+      <c r="CR44">
+        <v>-7.6999999999999999E-2</v>
+      </c>
+      <c r="CS44">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="CT44">
+        <v>0.2319</v>
+      </c>
+      <c r="CU44">
+        <v>-6.4899999999999999E-2</v>
+      </c>
+      <c r="CV44">
+        <v>-4.4999999999999997E-3</v>
+      </c>
+      <c r="CW44">
+        <v>0.92900000000000005</v>
+      </c>
+      <c r="CX44">
+        <v>-0.95030000000000003</v>
+      </c>
+      <c r="CY44">
+        <v>7.6769999999999996</v>
+      </c>
+      <c r="CZ44">
+        <v>8.0449999999999999</v>
+      </c>
+      <c r="DA44">
+        <v>10.3264</v>
+      </c>
+      <c r="DB44">
+        <v>27.045000000000002</v>
+      </c>
+      <c r="DC44">
+        <v>1</v>
+      </c>
+      <c r="DD44">
+        <v>1</v>
+      </c>
+      <c r="DE44">
+        <v>989.47410000000002</v>
+      </c>
+      <c r="DF44">
+        <v>1396.5781999999999</v>
+      </c>
+      <c r="DG44">
+        <v>888</v>
+      </c>
+      <c r="DH44">
+        <v>73.951599999999999</v>
+      </c>
+      <c r="DI44">
+        <v>0.1196</v>
+      </c>
+      <c r="DJ44">
+        <v>0</v>
+      </c>
+      <c r="DK44">
+        <v>8.0449999999999999</v>
+      </c>
+      <c r="DL44">
+        <v>83.014300000000006</v>
+      </c>
+      <c r="DM44">
+        <v>0</v>
+      </c>
+      <c r="DN44">
+        <v>0</v>
+      </c>
+      <c r="DO44">
+        <v>0</v>
+      </c>
+      <c r="DP44">
+        <v>7.0542999999999996</v>
+      </c>
+      <c r="DQ44">
+        <v>3.7694999999999999</v>
+      </c>
+      <c r="DR44">
+        <v>4.4581999999999997</v>
+      </c>
+      <c r="DS44">
+        <v>0.90310000000000001</v>
+      </c>
+      <c r="DT44">
+        <v>0.80059999999999998</v>
+      </c>
+      <c r="DU44">
+        <v>0</v>
+      </c>
+      <c r="DV44">
+        <v>0</v>
+      </c>
+      <c r="DW44">
+        <v>0</v>
+      </c>
+      <c r="DX44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>170</v>
+      </c>
+      <c r="B45" t="s">
+        <v>183</v>
+      </c>
+      <c r="C45" t="s">
+        <v>184</v>
+      </c>
+      <c r="D45" t="s">
+        <v>130</v>
+      </c>
+      <c r="BE45">
+        <v>31</v>
+      </c>
+      <c r="BI45">
+        <v>3420.5477999999998</v>
+      </c>
+      <c r="BK45">
+        <v>3420.5477999999998</v>
+      </c>
+      <c r="BM45">
+        <v>3420.5477999999998</v>
+      </c>
+      <c r="BO45">
+        <v>3420.5477999999998</v>
+      </c>
+      <c r="BQ45" s="2">
+        <v>3420.5477999999998</v>
+      </c>
+      <c r="BS45" s="10"/>
+      <c r="BY45">
+        <v>0</v>
+      </c>
+      <c r="BZ45">
+        <v>15.3355</v>
+      </c>
+      <c r="CA45">
+        <v>0.1321</v>
+      </c>
+      <c r="CB45">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="CC45">
+        <v>0</v>
+      </c>
+      <c r="CD45">
+        <v>0</v>
+      </c>
+      <c r="CI45">
+        <v>0</v>
+      </c>
+      <c r="CJ45">
+        <v>0</v>
+      </c>
+      <c r="CK45">
+        <v>0</v>
+      </c>
+      <c r="CL45">
+        <v>0</v>
+      </c>
+      <c r="CM45">
+        <v>0</v>
+      </c>
+      <c r="CN45">
+        <v>0</v>
+      </c>
+      <c r="CO45">
+        <v>0</v>
+      </c>
+      <c r="CP45">
+        <v>0</v>
+      </c>
+      <c r="CQ45">
+        <v>0</v>
+      </c>
+      <c r="CR45">
+        <v>0</v>
+      </c>
+      <c r="CS45">
+        <v>0</v>
+      </c>
+      <c r="CT45">
+        <v>0</v>
+      </c>
+      <c r="CU45">
+        <v>0</v>
+      </c>
+      <c r="CV45">
+        <v>0</v>
+      </c>
+      <c r="CW45">
+        <v>0</v>
+      </c>
+      <c r="CX45">
+        <v>0</v>
+      </c>
+      <c r="CY45">
+        <v>0</v>
+      </c>
+      <c r="CZ45">
+        <v>0</v>
+      </c>
+      <c r="DA45">
+        <v>0</v>
+      </c>
+      <c r="DB45">
+        <v>0</v>
+      </c>
+      <c r="DC45">
+        <v>0</v>
+      </c>
+      <c r="DD45">
+        <v>0</v>
+      </c>
+      <c r="DE45">
+        <v>1122.5806</v>
+      </c>
+      <c r="DF45">
+        <v>1200</v>
+      </c>
+      <c r="DH45">
+        <v>100</v>
+      </c>
+      <c r="DI45">
+        <v>0</v>
+      </c>
+      <c r="DJ45">
+        <v>0</v>
+      </c>
+      <c r="DK45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:128" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>174</v>
+      </c>
+      <c r="B46" t="s">
+        <v>186</v>
+      </c>
+      <c r="C46" t="s">
+        <v>187</v>
+      </c>
+      <c r="D46" t="s">
+        <v>130</v>
+      </c>
+      <c r="E46" t="s">
+        <v>131</v>
+      </c>
+      <c r="G46" t="s">
+        <v>132</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>14800</v>
+      </c>
+      <c r="J46">
+        <v>5170</v>
+      </c>
+      <c r="K46">
+        <v>19970</v>
+      </c>
+      <c r="L46" t="s">
+        <v>131</v>
+      </c>
+      <c r="M46" t="s">
+        <v>188</v>
+      </c>
+      <c r="N46" t="s">
+        <v>133</v>
+      </c>
+      <c r="O46">
+        <v>0</v>
+      </c>
+      <c r="P46">
+        <v>600</v>
+      </c>
+      <c r="Q46">
+        <v>0</v>
+      </c>
+      <c r="R46">
+        <v>7700</v>
+      </c>
+      <c r="S46">
+        <v>1</v>
+      </c>
+      <c r="T46">
+        <v>1</v>
+      </c>
+      <c r="U46">
+        <v>1</v>
+      </c>
+      <c r="V46">
+        <v>0</v>
+      </c>
+      <c r="W46">
+        <v>1</v>
+      </c>
+      <c r="X46">
+        <v>1</v>
+      </c>
+      <c r="Z46">
+        <v>4.1150000000000002</v>
+      </c>
+      <c r="AA46">
+        <v>6.65865774077144E-3</v>
+      </c>
+      <c r="AB46">
+        <v>6.65865774077144E-3</v>
+      </c>
+      <c r="AC46">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="AD46">
+        <v>1</v>
+      </c>
+      <c r="AE46">
+        <v>2</v>
+      </c>
+      <c r="AF46">
+        <v>0</v>
+      </c>
+      <c r="AG46" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH46" t="s">
+        <v>189</v>
+      </c>
+      <c r="AI46" t="s">
+        <v>135</v>
+      </c>
+      <c r="AJ46">
+        <v>3.36</v>
+      </c>
+      <c r="AK46">
+        <v>0.62</v>
+      </c>
+      <c r="AL46" t="s">
+        <v>136</v>
+      </c>
+      <c r="AM46" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN46" t="s">
+        <v>131</v>
+      </c>
+      <c r="AO46" t="s">
+        <v>132</v>
+      </c>
+      <c r="AP46" t="s">
+        <v>149</v>
+      </c>
+      <c r="AQ46" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR46" t="s">
+        <v>136</v>
+      </c>
+      <c r="AS46" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT46" t="s">
+        <v>131</v>
+      </c>
+      <c r="AU46" t="s">
+        <v>189</v>
+      </c>
+      <c r="AV46">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="BE46">
+        <v>13224.284900000001</v>
+      </c>
+      <c r="BF46">
+        <v>123.59</v>
+      </c>
+      <c r="BG46">
+        <v>33.644500000000001</v>
+      </c>
+      <c r="BH46">
+        <v>1.3106</v>
+      </c>
+      <c r="BI46">
+        <v>11853.2664</v>
+      </c>
+      <c r="BJ46">
+        <v>352.30950000000001</v>
+      </c>
+      <c r="BK46">
+        <v>11853.2664</v>
+      </c>
+      <c r="BL46">
+        <v>352.30950000000001</v>
+      </c>
+      <c r="BM46">
+        <v>11853.2664</v>
+      </c>
+      <c r="BN46">
+        <v>352.30950000000001</v>
+      </c>
+      <c r="BO46">
+        <v>11869.326300000001</v>
+      </c>
+      <c r="BP46">
+        <v>352.7869</v>
+      </c>
+      <c r="BQ46">
+        <v>11869.326300000001</v>
+      </c>
+      <c r="BR46">
+        <v>352.7869</v>
+      </c>
+      <c r="BS46" s="2">
+        <v>42.199399999999997</v>
+      </c>
+      <c r="BT46">
+        <v>8.1623999999999999</v>
+      </c>
+      <c r="BV46">
+        <v>1104.223</v>
+      </c>
+      <c r="BW46">
+        <v>213.58279999999999</v>
+      </c>
+      <c r="BY46">
+        <v>43.174300000000002</v>
+      </c>
+      <c r="BZ46">
+        <v>59.676299999999998</v>
+      </c>
+      <c r="CA46">
+        <v>219.21559999999999</v>
+      </c>
+      <c r="CB46">
+        <v>11.225</v>
+      </c>
+      <c r="CC46">
+        <v>0</v>
+      </c>
+      <c r="CD46">
+        <v>0</v>
+      </c>
+      <c r="CE46">
+        <v>18.367100000000001</v>
+      </c>
+      <c r="CI46">
+        <v>40.783999999999999</v>
+      </c>
+      <c r="CJ46">
+        <v>1.3601000000000001</v>
+      </c>
+      <c r="CK46">
+        <v>0</v>
+      </c>
+      <c r="CL46">
+        <v>0</v>
+      </c>
+      <c r="CM46">
+        <v>14.5189</v>
+      </c>
+      <c r="CN46">
+        <v>4.6505999999999998</v>
+      </c>
+      <c r="CO46">
+        <v>0</v>
+      </c>
+      <c r="CP46">
+        <v>15.077500000000001</v>
+      </c>
+      <c r="CQ46">
+        <v>64.801699999999997</v>
+      </c>
+      <c r="CR46">
+        <v>0</v>
+      </c>
+      <c r="CS46">
+        <v>22.033899999999999</v>
+      </c>
+      <c r="CT46">
+        <v>44.751899999999999</v>
+      </c>
+      <c r="CU46">
+        <v>1.12E-2</v>
+      </c>
+      <c r="CV46">
+        <v>0</v>
+      </c>
+      <c r="CW46">
+        <v>0.64829999999999999</v>
+      </c>
+      <c r="CX46">
+        <v>-0.70199999999999996</v>
+      </c>
+      <c r="CY46">
+        <v>20.511399999999998</v>
+      </c>
+      <c r="CZ46">
+        <v>18.125800000000002</v>
+      </c>
+      <c r="DA46">
+        <v>48.441099999999999</v>
+      </c>
+      <c r="DB46">
+        <v>84</v>
+      </c>
+      <c r="DC46">
+        <v>1</v>
+      </c>
+      <c r="DD46">
+        <v>1.3954</v>
+      </c>
+      <c r="DE46">
+        <v>1109.6643999999999</v>
+      </c>
+      <c r="DF46">
+        <v>1849.4880000000001</v>
+      </c>
+      <c r="DG46">
+        <v>863</v>
+      </c>
+      <c r="DH46">
+        <v>12.9217</v>
+      </c>
+      <c r="DI46">
+        <v>14.139799999999999</v>
+      </c>
+      <c r="DJ46">
+        <v>5.5111999999999997</v>
+      </c>
+      <c r="DK46">
+        <v>12.712300000000001</v>
+      </c>
+      <c r="DL46">
+        <v>23.465199999999999</v>
+      </c>
+      <c r="DM46">
+        <v>6.5080999999999998</v>
+      </c>
+      <c r="DN46">
+        <v>25.735399999999998</v>
+      </c>
+      <c r="DO46">
+        <v>8.9931000000000001</v>
+      </c>
+      <c r="DP46">
+        <v>15.617000000000001</v>
+      </c>
+      <c r="DQ46">
+        <v>10.132099999999999</v>
+      </c>
+      <c r="DR46">
+        <v>9.5490999999999993</v>
+      </c>
+    </row>
+    <row r="47" spans="1:128" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="8"/>
+    </row>
+    <row r="48" spans="1:128" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="8"/>
+      <c r="BS55" s="9"/>
+    </row>
+    <row r="56" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="BS56" s="9"/>
+    </row>
+    <row r="57" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="8"/>
+    </row>
+    <row r="58" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="8"/>
+      <c r="BS63" s="9"/>
+    </row>
+    <row r="64" spans="1:71" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="BS64" s="9"/>
+    </row>
+    <row r="65" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="8"/>
+    </row>
+    <row r="66" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="8"/>
+    </row>
+    <row r="71" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="8"/>
+    </row>
+    <row r="73" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>